<commit_message>
data: update Taiwan Lottery draws
</commit_message>
<xml_diff>
--- a/台灣彩券分析報告.xlsx
+++ b/台灣彩券分析報告.xlsx
@@ -31,7 +31,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>大樂透 2026-08-21 第 115000081 期；威力彩 2026-08-20 第 115000067 期</t>
+          <t>大樂透 2026-08-21 第 115000081 期；威力彩 2026-08-24 第 115000068 期</t>
         </is>
       </c>
     </row>
@@ -112,7 +112,7 @@
         </is>
       </c>
       <c r="C5">
-        <v>115000067</v>
+        <v>115000068</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -121,7 +121,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -143,7 +143,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>9, 11, 14, 29, 35, 38</t>
+          <t>9, 14, 29, 31, 35, 38</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -3508,7 +3508,7 @@
         <v>42</v>
       </c>
       <c r="C4">
-        <v>1.0</v>
+        <v>0.976</v>
       </c>
       <c r="D4">
         <v>23.8</v>
@@ -3523,7 +3523,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>均衡分散</t>
+          <t>冷號觀察</t>
         </is>
       </c>
       <c r="B5">
@@ -3533,10 +3533,10 @@
         <v>0.952</v>
       </c>
       <c r="D5">
-        <v>21.4</v>
+        <v>28.6</v>
       </c>
       <c r="E5">
-        <v>4.8</v>
+        <v>2.4</v>
       </c>
       <c r="F5">
         <v>3</v>
@@ -3545,20 +3545,20 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>冷號觀察</t>
+          <t>均衡分散</t>
         </is>
       </c>
       <c r="B6">
         <v>42</v>
       </c>
       <c r="C6">
-        <v>0.952</v>
+        <v>0.929</v>
       </c>
       <c r="D6">
-        <v>28.6</v>
+        <v>21.4</v>
       </c>
       <c r="E6">
-        <v>2.4</v>
+        <v>4.8</v>
       </c>
       <c r="F6">
         <v>3</v>
@@ -3648,25 +3648,25 @@
         <v>29</v>
       </c>
       <c r="C2">
-        <v>73.4</v>
+        <v>73.61</v>
       </c>
       <c r="D2">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E2">
         <v>6</v>
       </c>
       <c r="F2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G2">
-        <v>100.0</v>
+        <v>92.86</v>
       </c>
       <c r="H2">
         <v>100.0</v>
       </c>
       <c r="I2">
-        <v>0.0</v>
+        <v>3.03</v>
       </c>
     </row>
     <row r="3">
@@ -3674,28 +3674,28 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="C3">
-        <v>73.16</v>
+        <v>70.32</v>
       </c>
       <c r="D3">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E3">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F3">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G3">
-        <v>92.86</v>
+        <v>78.57</v>
       </c>
       <c r="H3">
-        <v>100.0</v>
+        <v>83.33</v>
       </c>
       <c r="I3">
-        <v>0.0</v>
+        <v>12.12</v>
       </c>
     </row>
     <row r="4">
@@ -3703,28 +3703,28 @@
         <v>3</v>
       </c>
       <c r="B4">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="C4">
-        <v>69.91</v>
+        <v>69.44</v>
       </c>
       <c r="D4">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E4">
         <v>5</v>
       </c>
       <c r="F4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G4">
-        <v>78.57</v>
+        <v>92.86</v>
       </c>
       <c r="H4">
         <v>83.33</v>
       </c>
       <c r="I4">
-        <v>9.38</v>
+        <v>3.03</v>
       </c>
     </row>
     <row r="5">
@@ -3732,28 +3732,28 @@
         <v>4</v>
       </c>
       <c r="B5">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="C5">
-        <v>68.5</v>
+        <v>65.38</v>
       </c>
       <c r="D5">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E5">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F5">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="G5">
-        <v>78.57</v>
+        <v>71.43</v>
       </c>
       <c r="H5">
-        <v>83.33</v>
+        <v>50.0</v>
       </c>
       <c r="I5">
-        <v>0.0</v>
+        <v>36.36</v>
       </c>
     </row>
     <row r="6">
@@ -3761,10 +3761,10 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="C6">
-        <v>66.44</v>
+        <v>65.01</v>
       </c>
       <c r="D6">
         <v>10</v>
@@ -3773,7 +3773,7 @@
         <v>4</v>
       </c>
       <c r="F6">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G6">
         <v>71.43</v>
@@ -3782,7 +3782,7 @@
         <v>66.67</v>
       </c>
       <c r="I6">
-        <v>15.62</v>
+        <v>6.06</v>
       </c>
     </row>
     <row r="7">
@@ -3790,28 +3790,28 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="C7">
-        <v>65.09</v>
+        <v>64.55</v>
       </c>
       <c r="D7">
         <v>10</v>
       </c>
       <c r="E7">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F7">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="G7">
         <v>71.43</v>
       </c>
       <c r="H7">
-        <v>50.0</v>
+        <v>66.67</v>
       </c>
       <c r="I7">
-        <v>34.38</v>
+        <v>3.03</v>
       </c>
     </row>
     <row r="8">
@@ -3819,28 +3819,28 @@
         <v>7</v>
       </c>
       <c r="B8">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="C8">
-        <v>64.56</v>
+        <v>63.61</v>
       </c>
       <c r="D8">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E8">
         <v>4</v>
       </c>
       <c r="F8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G8">
-        <v>71.43</v>
+        <v>57.14</v>
       </c>
       <c r="H8">
         <v>66.67</v>
       </c>
       <c r="I8">
-        <v>3.12</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="9">
@@ -3848,10 +3848,10 @@
         <v>8</v>
       </c>
       <c r="B9">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="C9">
-        <v>63.68</v>
+        <v>62.66</v>
       </c>
       <c r="D9">
         <v>10</v>
@@ -3860,7 +3860,7 @@
         <v>3</v>
       </c>
       <c r="F9">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G9">
         <v>71.43</v>
@@ -3869,7 +3869,7 @@
         <v>50.0</v>
       </c>
       <c r="I9">
-        <v>25.0</v>
+        <v>18.18</v>
       </c>
     </row>
     <row r="10">
@@ -3877,10 +3877,10 @@
         <v>9</v>
       </c>
       <c r="B10">
-        <v>21</v>
+        <v>8</v>
       </c>
       <c r="C10">
-        <v>62.25</v>
+        <v>61.71</v>
       </c>
       <c r="D10">
         <v>8</v>
@@ -3889,7 +3889,7 @@
         <v>3</v>
       </c>
       <c r="F10">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G10">
         <v>57.14</v>
@@ -3898,7 +3898,7 @@
         <v>50.0</v>
       </c>
       <c r="I10">
-        <v>18.75</v>
+        <v>15.15</v>
       </c>
     </row>
     <row r="11">
@@ -3906,10 +3906,10 @@
         <v>10</v>
       </c>
       <c r="B11">
-        <v>23</v>
+        <v>4</v>
       </c>
       <c r="C11">
-        <v>62.25</v>
+        <v>60.81</v>
       </c>
       <c r="D11">
         <v>8</v>
@@ -3918,7 +3918,7 @@
         <v>3</v>
       </c>
       <c r="F11">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G11">
         <v>57.14</v>
@@ -3927,7 +3927,7 @@
         <v>50.0</v>
       </c>
       <c r="I11">
-        <v>18.75</v>
+        <v>9.09</v>
       </c>
     </row>
     <row r="12">
@@ -3935,28 +3935,28 @@
         <v>11</v>
       </c>
       <c r="B12">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="C12">
-        <v>61.32</v>
+        <v>59.85</v>
       </c>
       <c r="D12">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E12">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F12">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="G12">
-        <v>57.14</v>
+        <v>71.43</v>
       </c>
       <c r="H12">
-        <v>50.0</v>
+        <v>33.33</v>
       </c>
       <c r="I12">
-        <v>12.5</v>
+        <v>27.27</v>
       </c>
     </row>
     <row r="13">
@@ -3964,10 +3964,10 @@
         <v>12</v>
       </c>
       <c r="B13">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C13">
-        <v>60.38</v>
+        <v>59.44</v>
       </c>
       <c r="D13">
         <v>8</v>
@@ -3976,7 +3976,7 @@
         <v>3</v>
       </c>
       <c r="F13">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G13">
         <v>57.14</v>
@@ -3985,7 +3985,7 @@
         <v>50.0</v>
       </c>
       <c r="I13">
-        <v>6.25</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="14">
@@ -3996,7 +3996,7 @@
         <v>34</v>
       </c>
       <c r="C14">
-        <v>58.35</v>
+        <v>58.73</v>
       </c>
       <c r="D14">
         <v>11</v>
@@ -4005,7 +4005,7 @@
         <v>2</v>
       </c>
       <c r="F14">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G14">
         <v>78.57</v>
@@ -4014,7 +4014,7 @@
         <v>33.33</v>
       </c>
       <c r="I14">
-        <v>15.62</v>
+        <v>18.18</v>
       </c>
     </row>
     <row r="15">
@@ -4025,7 +4025,7 @@
         <v>15</v>
       </c>
       <c r="C15">
-        <v>58.1</v>
+        <v>58.49</v>
       </c>
       <c r="D15">
         <v>10</v>
@@ -4034,7 +4034,7 @@
         <v>2</v>
       </c>
       <c r="F15">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G15">
         <v>71.43</v>
@@ -4043,7 +4043,7 @@
         <v>33.33</v>
       </c>
       <c r="I15">
-        <v>15.62</v>
+        <v>18.18</v>
       </c>
     </row>
     <row r="16">
@@ -4054,7 +4054,7 @@
         <v>17</v>
       </c>
       <c r="C16">
-        <v>58.09</v>
+        <v>58.46</v>
       </c>
       <c r="D16">
         <v>8</v>
@@ -4063,7 +4063,7 @@
         <v>2</v>
       </c>
       <c r="F16">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G16">
         <v>57.14</v>
@@ -4072,7 +4072,7 @@
         <v>33.33</v>
       </c>
       <c r="I16">
-        <v>18.75</v>
+        <v>21.21</v>
       </c>
     </row>
     <row r="17">
@@ -4080,28 +4080,28 @@
         <v>16</v>
       </c>
       <c r="B17">
-        <v>38</v>
+        <v>21</v>
       </c>
       <c r="C17">
-        <v>57.2</v>
+        <v>58.46</v>
       </c>
       <c r="D17">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="E17">
         <v>2</v>
       </c>
       <c r="F17">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="G17">
-        <v>100.0</v>
+        <v>57.14</v>
       </c>
       <c r="H17">
         <v>33.33</v>
       </c>
       <c r="I17">
-        <v>3.12</v>
+        <v>21.21</v>
       </c>
     </row>
     <row r="18">
@@ -4109,28 +4109,28 @@
         <v>17</v>
       </c>
       <c r="B18">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="C18">
-        <v>57.17</v>
+        <v>57.64</v>
       </c>
       <c r="D18">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="E18">
         <v>2</v>
       </c>
       <c r="F18">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G18">
-        <v>71.43</v>
+        <v>100.0</v>
       </c>
       <c r="H18">
         <v>33.33</v>
       </c>
       <c r="I18">
-        <v>9.38</v>
+        <v>6.06</v>
       </c>
     </row>
     <row r="19">
@@ -4138,13 +4138,13 @@
         <v>18</v>
       </c>
       <c r="B19">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="C19">
-        <v>57.15</v>
+        <v>57.58</v>
       </c>
       <c r="D19">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E19">
         <v>2</v>
@@ -4153,13 +4153,13 @@
         <v>4</v>
       </c>
       <c r="G19">
-        <v>57.14</v>
+        <v>71.43</v>
       </c>
       <c r="H19">
         <v>33.33</v>
       </c>
       <c r="I19">
-        <v>12.5</v>
+        <v>12.12</v>
       </c>
     </row>
     <row r="20">
@@ -4167,28 +4167,28 @@
         <v>19</v>
       </c>
       <c r="B20">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="C20">
-        <v>56.93</v>
+        <v>57.55</v>
       </c>
       <c r="D20">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E20">
         <v>2</v>
       </c>
       <c r="F20">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G20">
-        <v>64.29</v>
+        <v>57.14</v>
       </c>
       <c r="H20">
         <v>33.33</v>
       </c>
       <c r="I20">
-        <v>9.38</v>
+        <v>15.15</v>
       </c>
     </row>
     <row r="21">
@@ -4196,10 +4196,10 @@
         <v>20</v>
       </c>
       <c r="B21">
-        <v>7</v>
+        <v>25</v>
       </c>
       <c r="C21">
-        <v>56.21</v>
+        <v>57.09</v>
       </c>
       <c r="D21">
         <v>8</v>
@@ -4208,7 +4208,7 @@
         <v>2</v>
       </c>
       <c r="F21">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G21">
         <v>57.14</v>
@@ -4217,7 +4217,7 @@
         <v>33.33</v>
       </c>
       <c r="I21">
-        <v>6.25</v>
+        <v>12.12</v>
       </c>
     </row>
     <row r="22">
@@ -4225,28 +4225,28 @@
         <v>21</v>
       </c>
       <c r="B22">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="C22">
-        <v>54.65</v>
+        <v>56.49</v>
       </c>
       <c r="D22">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E22">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F22">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="G22">
-        <v>78.57</v>
+        <v>92.86</v>
       </c>
       <c r="H22">
-        <v>16.67</v>
+        <v>33.33</v>
       </c>
       <c r="I22">
-        <v>18.75</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="23">
@@ -4254,28 +4254,28 @@
         <v>22</v>
       </c>
       <c r="B23">
-        <v>27</v>
+        <v>36</v>
       </c>
       <c r="C23">
-        <v>54.26</v>
+        <v>55.93</v>
       </c>
       <c r="D23">
         <v>6</v>
       </c>
       <c r="E23">
+        <v>4</v>
+      </c>
+      <c r="F23">
         <v>0</v>
-      </c>
-      <c r="F23">
-        <v>32</v>
       </c>
       <c r="G23">
         <v>42.86</v>
       </c>
       <c r="H23">
+        <v>66.67</v>
+      </c>
+      <c r="I23">
         <v>0.0</v>
-      </c>
-      <c r="I23">
-        <v>100.0</v>
       </c>
     </row>
     <row r="24">
@@ -4283,28 +4283,28 @@
         <v>23</v>
       </c>
       <c r="B24">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="C24">
-        <v>52.7</v>
+        <v>55.27</v>
       </c>
       <c r="D24">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E24">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F24">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G24">
-        <v>42.86</v>
+        <v>57.14</v>
       </c>
       <c r="H24">
-        <v>50.0</v>
+        <v>33.33</v>
       </c>
       <c r="I24">
-        <v>6.25</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="25">
@@ -4312,28 +4312,28 @@
         <v>24</v>
       </c>
       <c r="B25">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="C25">
-        <v>52.33</v>
+        <v>55.02</v>
       </c>
       <c r="D25">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E25">
         <v>1</v>
       </c>
       <c r="F25">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="G25">
-        <v>92.86</v>
+        <v>78.57</v>
       </c>
       <c r="H25">
         <v>16.67</v>
       </c>
       <c r="I25">
-        <v>0.0</v>
+        <v>21.21</v>
       </c>
     </row>
     <row r="26">
@@ -4341,28 +4341,28 @@
         <v>25</v>
       </c>
       <c r="B26">
-        <v>2</v>
+        <v>27</v>
       </c>
       <c r="C26">
-        <v>51.76</v>
+        <v>54.26</v>
       </c>
       <c r="D26">
         <v>6</v>
       </c>
       <c r="E26">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F26">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="G26">
         <v>42.86</v>
       </c>
       <c r="H26">
-        <v>50.0</v>
+        <v>0.0</v>
       </c>
       <c r="I26">
-        <v>0.0</v>
+        <v>100.0</v>
       </c>
     </row>
     <row r="27">
@@ -4370,28 +4370,28 @@
         <v>26</v>
       </c>
       <c r="B27">
+        <v>10</v>
+      </c>
+      <c r="C27">
+        <v>53.12</v>
+      </c>
+      <c r="D27">
         <v>6</v>
       </c>
-      <c r="C27">
-        <v>51.69</v>
-      </c>
-      <c r="D27">
-        <v>7</v>
-      </c>
       <c r="E27">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F27">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="G27">
+        <v>42.86</v>
+      </c>
+      <c r="H27">
         <v>50.0</v>
       </c>
-      <c r="H27">
-        <v>16.67</v>
-      </c>
       <c r="I27">
-        <v>28.12</v>
+        <v>9.09</v>
       </c>
     </row>
     <row r="28">
@@ -4399,28 +4399,28 @@
         <v>27</v>
       </c>
       <c r="B28">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="C28">
-        <v>49.12</v>
+        <v>51.76</v>
       </c>
       <c r="D28">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E28">
         <v>3</v>
       </c>
       <c r="F28">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G28">
-        <v>35.71</v>
+        <v>42.86</v>
       </c>
       <c r="H28">
         <v>50.0</v>
       </c>
       <c r="I28">
-        <v>9.38</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="29">
@@ -4431,7 +4431,7 @@
         <v>32</v>
       </c>
       <c r="C29">
-        <v>48.58</v>
+        <v>48.88</v>
       </c>
       <c r="D29">
         <v>6</v>
@@ -4440,7 +4440,7 @@
         <v>1</v>
       </c>
       <c r="F29">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G29">
         <v>42.86</v>
@@ -4449,7 +4449,7 @@
         <v>16.67</v>
       </c>
       <c r="I29">
-        <v>34.38</v>
+        <v>36.36</v>
       </c>
     </row>
     <row r="30">
@@ -4460,7 +4460,7 @@
         <v>1</v>
       </c>
       <c r="C30">
-        <v>47.59</v>
+        <v>48.05</v>
       </c>
       <c r="D30">
         <v>6</v>
@@ -4469,7 +4469,7 @@
         <v>2</v>
       </c>
       <c r="F30">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G30">
         <v>42.86</v>
@@ -4478,7 +4478,7 @@
         <v>33.33</v>
       </c>
       <c r="I30">
-        <v>0.0</v>
+        <v>3.03</v>
       </c>
     </row>
     <row r="31">
@@ -4486,28 +4486,28 @@
         <v>30</v>
       </c>
       <c r="B31">
-        <v>26</v>
+        <v>2</v>
       </c>
       <c r="C31">
-        <v>45.42</v>
+        <v>48.05</v>
       </c>
       <c r="D31">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E31">
         <v>2</v>
       </c>
       <c r="F31">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G31">
-        <v>35.71</v>
+        <v>42.86</v>
       </c>
       <c r="H31">
         <v>33.33</v>
       </c>
       <c r="I31">
-        <v>12.5</v>
+        <v>3.03</v>
       </c>
     </row>
     <row r="32">
@@ -4518,7 +4518,7 @@
         <v>30</v>
       </c>
       <c r="C32">
-        <v>40.91</v>
+        <v>41.32</v>
       </c>
       <c r="D32">
         <v>4</v>
@@ -4527,7 +4527,7 @@
         <v>2</v>
       </c>
       <c r="F32">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G32">
         <v>28.57</v>
@@ -4536,7 +4536,7 @@
         <v>33.33</v>
       </c>
       <c r="I32">
-        <v>9.38</v>
+        <v>12.12</v>
       </c>
     </row>
     <row r="33">
@@ -4547,7 +4547,7 @@
         <v>5</v>
       </c>
       <c r="C33">
-        <v>39.85</v>
+        <v>40.29</v>
       </c>
       <c r="D33">
         <v>5</v>
@@ -4556,7 +4556,7 @@
         <v>1</v>
       </c>
       <c r="F33">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G33">
         <v>35.71</v>
@@ -4565,7 +4565,7 @@
         <v>16.67</v>
       </c>
       <c r="I33">
-        <v>3.12</v>
+        <v>6.06</v>
       </c>
     </row>
     <row r="34">
@@ -4576,7 +4576,7 @@
         <v>18</v>
       </c>
       <c r="C34">
-        <v>39.85</v>
+        <v>40.29</v>
       </c>
       <c r="D34">
         <v>5</v>
@@ -4585,7 +4585,7 @@
         <v>1</v>
       </c>
       <c r="F34">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G34">
         <v>35.71</v>
@@ -4594,7 +4594,7 @@
         <v>16.67</v>
       </c>
       <c r="I34">
-        <v>3.12</v>
+        <v>6.06</v>
       </c>
     </row>
     <row r="35">
@@ -4605,7 +4605,7 @@
         <v>12</v>
       </c>
       <c r="C35">
-        <v>39.68</v>
+        <v>40.01</v>
       </c>
       <c r="D35">
         <v>3</v>
@@ -4614,7 +4614,7 @@
         <v>2</v>
       </c>
       <c r="F35">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G35">
         <v>21.43</v>
@@ -4623,7 +4623,7 @@
         <v>33.33</v>
       </c>
       <c r="I35">
-        <v>28.12</v>
+        <v>30.3</v>
       </c>
     </row>
     <row r="36">
@@ -4634,7 +4634,7 @@
         <v>16</v>
       </c>
       <c r="C36">
-        <v>38.2</v>
+        <v>38.44</v>
       </c>
       <c r="D36">
         <v>4</v>
@@ -4643,7 +4643,7 @@
         <v>0</v>
       </c>
       <c r="F36">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G36">
         <v>28.57</v>
@@ -4652,7 +4652,7 @@
         <v>0.0</v>
       </c>
       <c r="I36">
-        <v>46.88</v>
+        <v>48.48</v>
       </c>
     </row>
     <row r="37">
@@ -4663,7 +4663,7 @@
         <v>3</v>
       </c>
       <c r="C37">
-        <v>36.28</v>
+        <v>36.7</v>
       </c>
       <c r="D37">
         <v>4</v>
@@ -4672,7 +4672,7 @@
         <v>1</v>
       </c>
       <c r="F37">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G37">
         <v>28.57</v>
@@ -4681,7 +4681,7 @@
         <v>16.67</v>
       </c>
       <c r="I37">
-        <v>6.25</v>
+        <v>9.09</v>
       </c>
     </row>
     <row r="38">
@@ -4692,7 +4692,7 @@
         <v>20</v>
       </c>
       <c r="C38">
-        <v>33.17</v>
+        <v>33.57</v>
       </c>
       <c r="D38">
         <v>3</v>
@@ -4701,7 +4701,7 @@
         <v>1</v>
       </c>
       <c r="F38">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G38">
         <v>21.43</v>
@@ -4710,7 +4710,7 @@
         <v>16.67</v>
       </c>
       <c r="I38">
-        <v>12.5</v>
+        <v>15.15</v>
       </c>
     </row>
     <row r="39">
@@ -4721,7 +4721,7 @@
         <v>37</v>
       </c>
       <c r="C39">
-        <v>32.88</v>
+        <v>33.16</v>
       </c>
       <c r="D39">
         <v>2</v>
@@ -4730,7 +4730,7 @@
         <v>1</v>
       </c>
       <c r="F39">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G39">
         <v>14.29</v>
@@ -4739,7 +4739,7 @@
         <v>16.67</v>
       </c>
       <c r="I39">
-        <v>37.5</v>
+        <v>39.39</v>
       </c>
     </row>
   </sheetData>
@@ -4798,216 +4798,216 @@
     </row>
     <row r="2">
       <c r="A2">
-        <v>115000067</v>
+        <v>115000068</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="C2">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D2">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="E2">
         <v>9</v>
       </c>
       <c r="F2">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="G2">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="H2">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="I2">
-        <v>2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3">
       <c r="A3">
-        <v>115000066</v>
+        <v>115000067</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="C3">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D3">
+        <v>2</v>
+      </c>
+      <c r="E3">
+        <v>9</v>
+      </c>
+      <c r="F3">
         <v>11</v>
       </c>
-      <c r="E3">
-        <v>18</v>
-      </c>
-      <c r="F3">
-        <v>19</v>
-      </c>
       <c r="G3">
+        <v>29</v>
+      </c>
+      <c r="H3">
         <v>35</v>
       </c>
-      <c r="H3">
-        <v>38</v>
-      </c>
       <c r="I3">
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4">
       <c r="A4">
-        <v>115000065</v>
+        <v>115000066</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="C4">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D4">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="E4">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="F4">
-        <v>7</v>
+        <v>19</v>
       </c>
       <c r="G4">
-        <v>10</v>
+        <v>35</v>
       </c>
       <c r="H4">
-        <v>19</v>
+        <v>38</v>
       </c>
       <c r="I4">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5">
       <c r="A5">
-        <v>115000064</v>
+        <v>115000065</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="C5">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="D5">
-        <v>25</v>
+        <v>3</v>
       </c>
       <c r="E5">
-        <v>28</v>
+        <v>4</v>
       </c>
       <c r="F5">
-        <v>30</v>
+        <v>7</v>
       </c>
       <c r="G5">
-        <v>31</v>
+        <v>10</v>
       </c>
       <c r="H5">
-        <v>36</v>
+        <v>19</v>
       </c>
       <c r="I5">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6">
       <c r="A6">
-        <v>115000063</v>
+        <v>115000064</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="C6">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="D6">
-        <v>7</v>
+        <v>25</v>
       </c>
       <c r="E6">
-        <v>8</v>
+        <v>28</v>
       </c>
       <c r="F6">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="G6">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="H6">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="I6">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7">
       <c r="A7">
-        <v>115000062</v>
+        <v>115000063</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="C7">
+        <v>2</v>
+      </c>
+      <c r="D7">
+        <v>7</v>
+      </c>
+      <c r="E7">
+        <v>8</v>
+      </c>
+      <c r="F7">
+        <v>20</v>
+      </c>
+      <c r="G7">
+        <v>26</v>
+      </c>
+      <c r="H7">
+        <v>33</v>
+      </c>
+      <c r="I7">
         <v>4</v>
-      </c>
-      <c r="D7">
-        <v>15</v>
-      </c>
-      <c r="E7">
-        <v>22</v>
-      </c>
-      <c r="F7">
-        <v>26</v>
-      </c>
-      <c r="G7">
-        <v>34</v>
-      </c>
-      <c r="H7">
-        <v>36</v>
-      </c>
-      <c r="I7">
-        <v>7</v>
       </c>
     </row>
     <row r="8">
       <c r="A8">
-        <v>115000061</v>
+        <v>115000062</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="C8">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D8">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E8">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="F8">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="G8">
-        <v>21</v>
+        <v>34</v>
       </c>
       <c r="H8">
-        <v>23</v>
+        <v>36</v>
       </c>
       <c r="I8">
         <v>7</v>
@@ -5015,30 +5015,30 @@
     </row>
     <row r="9">
       <c r="A9">
-        <v>115000060</v>
+        <v>115000061</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="C9">
+        <v>8</v>
+      </c>
+      <c r="D9">
+        <v>14</v>
+      </c>
+      <c r="E9">
+        <v>17</v>
+      </c>
+      <c r="F9">
         <v>19</v>
       </c>
-      <c r="D9">
-        <v>22</v>
-      </c>
-      <c r="E9">
-        <v>28</v>
-      </c>
-      <c r="F9">
-        <v>31</v>
-      </c>
       <c r="G9">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="H9">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="I9">
         <v>7</v>
@@ -5046,30 +5046,30 @@
     </row>
     <row r="10">
       <c r="A10">
-        <v>115000059</v>
+        <v>115000060</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="C10">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="D10">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="E10">
-        <v>13</v>
+        <v>28</v>
       </c>
       <c r="F10">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="G10">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="H10">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="I10">
         <v>7</v>
@@ -5077,24 +5077,24 @@
     </row>
     <row r="11">
       <c r="A11">
-        <v>115000058</v>
+        <v>115000059</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="C11">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D11">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E11">
         <v>13</v>
       </c>
       <c r="F11">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="G11">
         <v>29</v>
@@ -5103,97 +5103,97 @@
         <v>31</v>
       </c>
       <c r="I11">
-        <v>2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="12">
       <c r="A12">
-        <v>115000057</v>
+        <v>115000058</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="C12">
-        <v>17</v>
+        <v>6</v>
       </c>
       <c r="D12">
+        <v>12</v>
+      </c>
+      <c r="E12">
+        <v>13</v>
+      </c>
+      <c r="F12">
         <v>23</v>
       </c>
-      <c r="E12">
-        <v>25</v>
-      </c>
-      <c r="F12">
+      <c r="G12">
         <v>29</v>
       </c>
-      <c r="G12">
-        <v>34</v>
-      </c>
       <c r="H12">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="I12">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13">
       <c r="A13">
-        <v>115000056</v>
+        <v>115000057</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="C13">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="D13">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E13">
+        <v>25</v>
+      </c>
+      <c r="F13">
         <v>29</v>
       </c>
-      <c r="F13">
-        <v>32</v>
-      </c>
       <c r="G13">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="H13">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="I13">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="14">
       <c r="A14">
-        <v>115000055</v>
+        <v>115000056</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="C14">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D14">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="E14">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="F14">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="G14">
         <v>35</v>
       </c>
       <c r="H14">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="I14">
         <v>6</v>
@@ -5201,402 +5201,402 @@
     </row>
     <row r="15">
       <c r="A15">
-        <v>115000054</v>
+        <v>115000055</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="C15">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="D15">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="E15">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="F15">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="G15">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="H15">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="I15">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="16">
       <c r="A16">
-        <v>115000053</v>
+        <v>115000054</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C16">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D16">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E16">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F16">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="G16">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="H16">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="I16">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17">
       <c r="A17">
-        <v>115000052</v>
+        <v>115000053</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="C17">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D17">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="E17">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="F17">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="G17">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="H17">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="I17">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="18">
       <c r="A18">
-        <v>115000051</v>
+        <v>115000052</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="C18">
+        <v>5</v>
+      </c>
+      <c r="D18">
         <v>6</v>
       </c>
-      <c r="D18">
-        <v>10</v>
-      </c>
       <c r="E18">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="F18">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="G18">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="H18">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="I18">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="19">
       <c r="A19">
-        <v>115000050</v>
+        <v>115000051</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="C19">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="D19">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="E19">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="F19">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="G19">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="H19">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="I19">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20">
       <c r="A20">
-        <v>115000049</v>
+        <v>115000050</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C20">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="D20">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="E20">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="F20">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="G20">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="H20">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I20">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="21">
       <c r="A21">
-        <v>115000048</v>
+        <v>115000049</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="C21">
+        <v>2</v>
+      </c>
+      <c r="D21">
+        <v>8</v>
+      </c>
+      <c r="E21">
+        <v>9</v>
+      </c>
+      <c r="F21">
+        <v>15</v>
+      </c>
+      <c r="G21">
+        <v>18</v>
+      </c>
+      <c r="H21">
+        <v>23</v>
+      </c>
+      <c r="I21">
         <v>4</v>
-      </c>
-      <c r="D21">
-        <v>17</v>
-      </c>
-      <c r="E21">
-        <v>19</v>
-      </c>
-      <c r="F21">
-        <v>25</v>
-      </c>
-      <c r="G21">
-        <v>28</v>
-      </c>
-      <c r="H21">
-        <v>29</v>
-      </c>
-      <c r="I21">
-        <v>6</v>
       </c>
     </row>
     <row r="22">
       <c r="A22">
-        <v>115000047</v>
+        <v>115000048</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="C22">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D22">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="E22">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="F22">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G22">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="H22">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="I22">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="23">
       <c r="A23">
-        <v>115000046</v>
+        <v>115000047</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="C23">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D23">
-        <v>7</v>
+        <v>22</v>
       </c>
       <c r="E23">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="F23">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="G23">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="H23">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="I23">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="24">
       <c r="A24">
-        <v>115000045</v>
+        <v>115000046</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="C24">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="D24">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="E24">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="F24">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="G24">
         <v>28</v>
       </c>
       <c r="H24">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="I24">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="25">
       <c r="A25">
-        <v>115000044</v>
+        <v>115000045</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="C25">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D25">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="E25">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="F25">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="G25">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="H25">
         <v>35</v>
       </c>
       <c r="I25">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="26">
       <c r="A26">
-        <v>115000043</v>
+        <v>115000044</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="C26">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D26">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="E26">
+        <v>9</v>
+      </c>
+      <c r="F26">
+        <v>15</v>
+      </c>
+      <c r="G26">
         <v>24</v>
       </c>
-      <c r="F26">
-        <v>31</v>
-      </c>
-      <c r="G26">
-        <v>34</v>
-      </c>
       <c r="H26">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="I26">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="27">
       <c r="A27">
-        <v>115000042</v>
+        <v>115000043</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="C27">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D27">
-        <v>17</v>
+        <v>2</v>
       </c>
       <c r="E27">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="F27">
-        <v>24</v>
+        <v>31</v>
       </c>
       <c r="G27">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="H27">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="I27">
         <v>3</v>
@@ -5604,554 +5604,554 @@
     </row>
     <row r="28">
       <c r="A28">
-        <v>115000041</v>
+        <v>115000042</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="C28">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D28">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E28">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F28">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="G28">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="H28">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="I28">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="29">
       <c r="A29">
-        <v>115000040</v>
+        <v>115000041</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="C29">
         <v>6</v>
       </c>
       <c r="D29">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="E29">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="F29">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="G29">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="H29">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="I29">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="30">
       <c r="A30">
-        <v>115000039</v>
+        <v>115000040</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="C30">
         <v>6</v>
       </c>
       <c r="D30">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E30">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="F30">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="G30">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="H30">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="I30">
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="31">
       <c r="A31">
-        <v>115000038</v>
+        <v>115000039</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="C31">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="D31">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="E31">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="F31">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="G31">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="H31">
-        <v>38</v>
+        <v>29</v>
       </c>
       <c r="I31">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="32">
       <c r="A32">
-        <v>115000037</v>
+        <v>115000038</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="C32">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="D32">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="E32">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="F32">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="G32">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="H32">
         <v>38</v>
       </c>
       <c r="I32">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="33">
       <c r="A33">
-        <v>115000036</v>
+        <v>115000037</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="C33">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D33">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="E33">
-        <v>29</v>
+        <v>15</v>
       </c>
       <c r="F33">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="G33">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="H33">
         <v>38</v>
       </c>
       <c r="I33">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="34">
       <c r="A34">
-        <v>115000035</v>
+        <v>115000036</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="C34">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D34">
-        <v>4</v>
+        <v>21</v>
       </c>
       <c r="E34">
-        <v>13</v>
+        <v>29</v>
       </c>
       <c r="F34">
-        <v>19</v>
+        <v>32</v>
       </c>
       <c r="G34">
-        <v>27</v>
+        <v>36</v>
       </c>
       <c r="H34">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="I34">
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="35">
       <c r="A35">
-        <v>115000034</v>
+        <v>115000035</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="C35">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="D35">
+        <v>4</v>
+      </c>
+      <c r="E35">
+        <v>13</v>
+      </c>
+      <c r="F35">
+        <v>19</v>
+      </c>
+      <c r="G35">
+        <v>27</v>
+      </c>
+      <c r="H35">
+        <v>30</v>
+      </c>
+      <c r="I35">
         <v>8</v>
-      </c>
-      <c r="E35">
-        <v>27</v>
-      </c>
-      <c r="F35">
-        <v>33</v>
-      </c>
-      <c r="G35">
-        <v>35</v>
-      </c>
-      <c r="H35">
-        <v>38</v>
-      </c>
-      <c r="I35">
-        <v>2</v>
       </c>
     </row>
     <row r="36">
       <c r="A36">
-        <v>115000033</v>
+        <v>115000034</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="C36">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D36">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="E36">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="F36">
-        <v>16</v>
+        <v>33</v>
       </c>
       <c r="G36">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="H36">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="I36">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="37">
       <c r="A37">
-        <v>115000032</v>
+        <v>115000033</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-23</t>
         </is>
       </c>
       <c r="C37">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="D37">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E37">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="F37">
-        <v>34</v>
+        <v>16</v>
       </c>
       <c r="G37">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="H37">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="I37">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="38">
       <c r="A38">
-        <v>115000031</v>
+        <v>115000032</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="C38">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D38">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E38">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="F38">
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="G38">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="H38">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I38">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="39">
       <c r="A39">
-        <v>115000030</v>
+        <v>115000031</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="C39">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D39">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E39">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="F39">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="G39">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="H39">
-        <v>24</v>
+        <v>38</v>
       </c>
       <c r="I39">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="40">
       <c r="A40">
-        <v>115000029</v>
+        <v>115000030</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="C40">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D40">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E40">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F40">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="G40">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="H40">
-        <v>34</v>
+        <v>24</v>
       </c>
       <c r="I40">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="41">
       <c r="A41">
-        <v>115000028</v>
+        <v>115000029</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="C41">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D41">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E41">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="F41">
         <v>27</v>
       </c>
       <c r="G41">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="H41">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="I41">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="42">
       <c r="A42">
-        <v>115000027</v>
+        <v>115000028</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="C42">
         <v>5</v>
       </c>
       <c r="D42">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="E42">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="F42">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="G42">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="H42">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="I42">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="43">
       <c r="A43">
-        <v>115000026</v>
+        <v>115000027</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="C43">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D43">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E43">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="F43">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G43">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="H43">
         <v>34</v>
       </c>
       <c r="I43">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="44">
       <c r="A44">
-        <v>115000025</v>
+        <v>115000026</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="C44">
+        <v>2</v>
+      </c>
+      <c r="D44">
         <v>13</v>
       </c>
-      <c r="D44">
-        <v>14</v>
-      </c>
       <c r="E44">
+        <v>21</v>
+      </c>
+      <c r="F44">
         <v>22</v>
       </c>
-      <c r="F44">
-        <v>28</v>
-      </c>
       <c r="G44">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="H44">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="I44">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="45">
       <c r="A45">
-        <v>115000024</v>
+        <v>115000025</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="C45">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="D45">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="E45">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="F45">
         <v>28</v>
       </c>
       <c r="G45">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="H45">
         <v>38</v>
@@ -6162,58 +6162,58 @@
     </row>
     <row r="46">
       <c r="A46">
-        <v>115000023</v>
+        <v>115000024</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-23</t>
         </is>
       </c>
       <c r="C46">
+        <v>1</v>
+      </c>
+      <c r="D46">
         <v>9</v>
       </c>
-      <c r="D46">
-        <v>13</v>
-      </c>
       <c r="E46">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="F46">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="G46">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="H46">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="I46">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="47">
       <c r="A47">
-        <v>115000022</v>
+        <v>115000023</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="C47">
+        <v>9</v>
+      </c>
+      <c r="D47">
+        <v>13</v>
+      </c>
+      <c r="E47">
         <v>14</v>
       </c>
-      <c r="D47">
-        <v>26</v>
-      </c>
-      <c r="E47">
-        <v>28</v>
-      </c>
       <c r="F47">
+        <v>18</v>
+      </c>
+      <c r="G47">
         <v>31</v>
-      </c>
-      <c r="G47">
-        <v>32</v>
       </c>
       <c r="H47">
         <v>34</v>
@@ -6224,61 +6224,61 @@
     </row>
     <row r="48">
       <c r="A48">
-        <v>115000021</v>
+        <v>115000022</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-03-16</t>
         </is>
       </c>
       <c r="C48">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="D48">
-        <v>9</v>
+        <v>26</v>
       </c>
       <c r="E48">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="F48">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="G48">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="H48">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="I48">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="49">
       <c r="A49">
-        <v>115000020</v>
+        <v>115000021</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-03-09</t>
+          <t>2026-03-12</t>
         </is>
       </c>
       <c r="C49">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D49">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E49">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F49">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="G49">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="H49">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="I49">
         <v>8</v>
@@ -6286,15 +6286,15 @@
     </row>
     <row r="50">
       <c r="A50">
-        <v>115000019</v>
+        <v>115000020</v>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-03-09</t>
         </is>
       </c>
       <c r="C50">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="D50">
         <v>11</v>
@@ -6303,47 +6303,47 @@
         <v>14</v>
       </c>
       <c r="F50">
+        <v>17</v>
+      </c>
+      <c r="G50">
+        <v>29</v>
+      </c>
+      <c r="H50">
         <v>32</v>
       </c>
-      <c r="G50">
-        <v>36</v>
-      </c>
-      <c r="H50">
-        <v>38</v>
-      </c>
       <c r="I50">
-        <v>2</v>
+        <v>8</v>
       </c>
     </row>
     <row r="51">
       <c r="A51">
-        <v>115000018</v>
+        <v>115000019</v>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-03-02</t>
+          <t>2026-03-05</t>
         </is>
       </c>
       <c r="C51">
         <v>7</v>
       </c>
       <c r="D51">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E51">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="F51">
-        <v>23</v>
+        <v>32</v>
       </c>
       <c r="G51">
-        <v>25</v>
+        <v>36</v>
       </c>
       <c r="H51">
-        <v>29</v>
+        <v>38</v>
       </c>
       <c r="I51">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>